<commit_message>
CORRECCION TOTAL Y NUEVO VISUAL
</commit_message>
<xml_diff>
--- a/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
+++ b/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
@@ -413,23 +413,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BASE</t>
+          <t>HOJA</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>TABLA</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>REGISTROS</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>COLUMNAS</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -441,14 +441,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VENTA</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>149999</v>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>campo_indicadores</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>14</v>
+        <v>188</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -459,14 +461,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PARTICIPACION</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>79290</v>
+          <t>Liquidacion por Rutas</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>campo_liquidacion_rutas</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>17</v>
+        <v>188</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -477,88 +481,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MERCADERISTA</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7441</v>
+          <t>Liquidacion Lideres y Superviso</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>campo_liquidacion_lideres</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>FECHAS CORTAS</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>8432</v>
-      </c>
-      <c r="C5" t="n">
-        <v>19</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DEVOLUCIONES</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>43511</v>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>COBERTURA</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2183</v>
-      </c>
-      <c r="C7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AGOTADOS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>119755</v>
-      </c>
-      <c r="C8" t="n">
-        <v>15</v>
-      </c>
-      <c r="D8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>

<commit_message>
ACT BASE DE DATOS
</commit_message>
<xml_diff>
--- a/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
+++ b/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
@@ -445,11 +445,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>376</v>
+        <v>564</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,11 +465,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>376</v>
+        <v>564</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -505,11 +505,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">

</xml_diff>

<commit_message>
ACT COMISIONES 22 OCT
</commit_message>
<xml_diff>
--- a/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
+++ b/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
@@ -445,11 +445,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>752</v>
+        <v>564</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,11 +465,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>752</v>
+        <v>564</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -485,11 +485,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>752</v>
+        <v>564</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -505,11 +505,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -525,11 +525,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -545,11 +545,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
ACT COMISIONES NEW 22 OCT
</commit_message>
<xml_diff>
--- a/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
+++ b/BASE DE DATOS/CONTROL_EXTRACCION.xlsx
@@ -445,11 +445,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>564</v>
+        <v>752</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,11 +465,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>564</v>
+        <v>752</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -485,11 +485,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>564</v>
+        <v>752</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -505,11 +505,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -525,11 +525,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -545,11 +545,11 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Agosto 2026, Julio 2026, Septiembre 2026</t>
+          <t>Agosto 2026, Julio 2026, Octubre 2026, Septiembre 2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>